<commit_message>
Git sh to ease commit and push
</commit_message>
<xml_diff>
--- a/controlRoom_server/server/templates/ICR_TEMPLATE016.xlsx
+++ b/controlRoom_server/server/templates/ICR_TEMPLATE016.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF7F0F1-980B-B348-8ADD-743DD04114E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E16856C8-5ACA-1044-AAF0-1A7C1DB0823D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="16400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,14 +11,27 @@
     <sheet name="ICR_TEMPLATE016.xlsx" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ICR_TEMPLATE016.xlsx!$A$1:$G$7</definedName>
+    <definedName name="_xlnm._FilterDatabase">ICR_TEMPLATE016.xlsx!$A$1:$H$7</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>UPC</t>
   </si>
@@ -29,43 +42,56 @@
     <t>SCHEMATIC</t>
   </si>
   <si>
+    <t>EFFECTIVE_DATE</t>
+  </si>
+  <si>
+    <t>SHELF_NUMBER</t>
+  </si>
+  <si>
+    <t>LOCATION_NUMBER</t>
+  </si>
+  <si>
     <t>CAPACITY</t>
   </si>
   <si>
     <t>FACING</t>
   </si>
   <si>
+    <t>10668074084</t>
+  </si>
+  <si>
+    <t>10668075029</t>
+  </si>
+  <si>
+    <t>10668075197</t>
+  </si>
+  <si>
+    <t>10668075241</t>
+  </si>
+  <si>
+    <t>10900000185</t>
+  </si>
+  <si>
     <t>10900005043</t>
   </si>
   <si>
-    <t>10900000185</t>
-  </si>
-  <si>
-    <t>10668075029</t>
-  </si>
-  <si>
-    <t>10668075241</t>
-  </si>
-  <si>
-    <t>10668074084</t>
-  </si>
-  <si>
-    <t>10668075197</t>
-  </si>
-  <si>
-    <t>SHELF_NUMBER</t>
-  </si>
-  <si>
-    <t>LOCATION_NUMBER</t>
+    <t>11/10/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -134,27 +160,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -471,21 +500,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="12.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20" style="2" customWidth="1"/>
+    <col min="6" max="6" width="23.5" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14" style="3" customWidth="1"/>
+    <col min="8" max="8" width="12.5" style="2" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -495,163 +525,180 @@
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>11</v>
+      <c r="D1" s="9" t="s">
+        <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="7">
+        <v>10</v>
+      </c>
+      <c r="C2" s="8">
+        <v>12118</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7">
         <v>12</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>4</v>
+      <c r="G2" s="8">
+        <v>5</v>
+      </c>
+      <c r="H2" s="8">
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+    <row r="3" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B3" s="7">
         <v>10</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C3" s="8">
         <v>12118</v>
       </c>
-      <c r="D2" s="8">
-        <v>1</v>
-      </c>
-      <c r="E2" s="8">
-        <v>12</v>
-      </c>
-      <c r="F2" s="7">
+      <c r="D3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="7">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7">
+        <v>15</v>
+      </c>
+      <c r="G3" s="8">
         <v>5</v>
       </c>
-      <c r="G2" s="7">
+      <c r="H3" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="9">
-        <v>10</v>
-      </c>
-      <c r="C3" s="7">
-        <v>12118</v>
-      </c>
-      <c r="D3" s="8">
-        <v>1</v>
-      </c>
-      <c r="E3" s="8">
-        <v>15</v>
-      </c>
-      <c r="F3" s="7">
-        <v>5</v>
-      </c>
-      <c r="G3" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="7">
         <v>10</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="8">
         <v>12118</v>
       </c>
-      <c r="D4" s="8">
-        <v>1</v>
-      </c>
-      <c r="E4" s="8">
+      <c r="D4" s="10" t="s">
         <v>14</v>
       </c>
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
       <c r="F4" s="7">
+        <v>14</v>
+      </c>
+      <c r="G4" s="8">
         <v>5</v>
       </c>
-      <c r="G4" s="7">
+      <c r="H4" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="9">
+        <v>11</v>
+      </c>
+      <c r="B5" s="7">
         <v>10</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="8">
         <v>12118</v>
       </c>
-      <c r="D5" s="8">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8">
+      <c r="D5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="7">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7">
         <v>11</v>
       </c>
-      <c r="F5" s="7">
+      <c r="G5" s="8">
         <v>6</v>
       </c>
-      <c r="G5" s="7">
+      <c r="H5" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="9">
+        <v>12</v>
+      </c>
+      <c r="B6" s="7">
         <v>10</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="8">
         <v>10569</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="7">
         <v>3</v>
       </c>
-      <c r="E6" s="8">
-        <v>1</v>
-      </c>
       <c r="F6" s="7">
+        <v>1</v>
+      </c>
+      <c r="G6" s="8">
         <v>32</v>
       </c>
-      <c r="G6" s="7">
+      <c r="H6" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="7">
+        <v>10</v>
+      </c>
+      <c r="C7" s="8">
+        <v>10569</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="7">
+        <v>7</v>
+      </c>
+      <c r="F7" s="7">
         <v>5</v>
       </c>
-      <c r="B7" s="9">
-        <v>10</v>
-      </c>
-      <c r="C7" s="7">
-        <v>10569</v>
-      </c>
-      <c r="D7" s="8">
-        <v>7</v>
-      </c>
-      <c r="E7" s="8">
-        <v>5</v>
-      </c>
-      <c r="F7" s="7">
+      <c r="G7" s="8">
         <v>36</v>
       </c>
-      <c r="G7" s="7">
+      <c r="H7" s="8">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G7" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G7">
-      <sortCondition ref="A1:A7"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:H7" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>